<commit_message>
CD3 Automation Toolkit v2026.2.0
</commit_message>
<xml_diff>
--- a/cd3_automation_toolkit/example/CD3-Azure-template.xlsx
+++ b/cd3_automation_toolkit/example/CD3-Azure-template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10621"/>
   <workbookPr updateLinks="never" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/susingla/PycharmProjects/orahub-develop/cd3_automation_toolkit/example/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B020AF44-9EAB-B442-B5EF-65782E103F6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{106C4731-84FE-0A4A-9F63-F9F5FA6A0484}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3960" yWindow="3000" windowWidth="30240" windowHeight="17440" tabRatio="1000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1587,51 +1587,6 @@
     <t>Customer Contacts</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>CD3 Automation Toolkit</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Release - v2025.2.0</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-  </si>
-  <si>
     <t>abc@yahoo.com,def@gmail.com</t>
   </si>
   <si>
@@ -2009,6 +1964,51 @@
   </si>
   <si>
     <t>vmname2</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>CD3 Automation Toolkit</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Release - v2026.2.0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -4432,7 +4432,7 @@
     <row r="1" spans="1:1" ht="16" thickBot="1"/>
     <row r="2" spans="1:1" ht="59.25" customHeight="1" thickBot="1">
       <c r="A2" s="36" t="s">
-        <v>471</v>
+        <v>541</v>
       </c>
     </row>
   </sheetData>
@@ -4464,7 +4464,7 @@
   <sheetData>
     <row r="1" spans="1:20" ht="79" customHeight="1">
       <c r="A1" s="57" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="B1" s="57"/>
       <c r="C1" s="57"/>
@@ -4491,16 +4491,16 @@
         <v>0</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="C2" s="7" t="s">
         <v>180</v>
       </c>
       <c r="D2" s="7" t="s">
+        <v>529</v>
+      </c>
+      <c r="E2" s="7" t="s">
         <v>530</v>
-      </c>
-      <c r="E2" s="7" t="s">
-        <v>531</v>
       </c>
       <c r="F2" s="7" t="s">
         <v>110</v>
@@ -4550,19 +4550,19 @@
     </row>
     <row r="3" spans="1:20" ht="63" customHeight="1">
       <c r="A3" s="24" t="s">
+        <v>527</v>
+      </c>
+      <c r="B3" s="24" t="s">
         <v>528</v>
-      </c>
-      <c r="B3" s="24" t="s">
-        <v>529</v>
       </c>
       <c r="C3" s="24" t="s">
         <v>182</v>
       </c>
       <c r="D3" s="25" t="s">
+        <v>532</v>
+      </c>
+      <c r="E3" s="25" t="s">
         <v>533</v>
-      </c>
-      <c r="E3" s="25" t="s">
-        <v>534</v>
       </c>
       <c r="F3" s="24" t="s">
         <v>468</v>
@@ -4604,10 +4604,10 @@
         <v>0</v>
       </c>
       <c r="S3" s="25" t="s">
+        <v>471</v>
+      </c>
+      <c r="T3" s="25" t="s">
         <v>472</v>
-      </c>
-      <c r="T3" s="25" t="s">
-        <v>473</v>
       </c>
     </row>
     <row r="4" spans="1:20">
@@ -4692,7 +4692,7 @@
   <sheetData>
     <row r="1" spans="1:18" ht="20" customHeight="1">
       <c r="A1" s="58" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="B1" s="57"/>
       <c r="C1" s="57"/>
@@ -4717,49 +4717,49 @@
         <v>0</v>
       </c>
       <c r="B2" s="47" t="s">
+        <v>473</v>
+      </c>
+      <c r="C2" s="48" t="s">
         <v>474</v>
       </c>
-      <c r="C2" s="48" t="s">
+      <c r="D2" s="47" t="s">
         <v>475</v>
-      </c>
-      <c r="D2" s="47" t="s">
-        <v>476</v>
       </c>
       <c r="E2" s="47" t="s">
         <v>14</v>
       </c>
       <c r="F2" s="47" t="s">
+        <v>476</v>
+      </c>
+      <c r="G2" s="47" t="s">
         <v>477</v>
       </c>
-      <c r="G2" s="47" t="s">
+      <c r="H2" s="47" t="s">
         <v>478</v>
       </c>
-      <c r="H2" s="47" t="s">
+      <c r="I2" s="47" t="s">
         <v>479</v>
       </c>
-      <c r="I2" s="47" t="s">
+      <c r="J2" s="47" t="s">
         <v>480</v>
       </c>
-      <c r="J2" s="47" t="s">
+      <c r="K2" s="47" t="s">
         <v>481</v>
       </c>
-      <c r="K2" s="47" t="s">
+      <c r="L2" s="47" t="s">
         <v>482</v>
       </c>
-      <c r="L2" s="47" t="s">
+      <c r="M2" s="47" t="s">
         <v>483</v>
       </c>
-      <c r="M2" s="47" t="s">
+      <c r="N2" s="47" t="s">
         <v>484</v>
       </c>
-      <c r="N2" s="47" t="s">
+      <c r="O2" s="47" t="s">
         <v>485</v>
       </c>
-      <c r="O2" s="47" t="s">
+      <c r="P2" s="47" t="s">
         <v>486</v>
-      </c>
-      <c r="P2" s="47" t="s">
-        <v>487</v>
       </c>
       <c r="Q2" s="47" t="s">
         <v>470</v>
@@ -4773,16 +4773,16 @@
         <v>467</v>
       </c>
       <c r="B3" s="24" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="C3" s="38" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D3" s="24">
         <v>1</v>
       </c>
       <c r="E3" s="38" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="F3" s="25">
         <v>2</v>
@@ -4791,37 +4791,37 @@
         <v>3</v>
       </c>
       <c r="H3" s="24" t="s">
+        <v>489</v>
+      </c>
+      <c r="I3" s="24" t="s">
         <v>490</v>
       </c>
-      <c r="I3" s="24" t="s">
+      <c r="J3" s="24" t="s">
         <v>491</v>
       </c>
-      <c r="J3" s="24" t="s">
+      <c r="K3" s="24" t="s">
         <v>492</v>
       </c>
-      <c r="K3" s="24" t="s">
+      <c r="L3" s="24" t="s">
         <v>493</v>
-      </c>
-      <c r="L3" s="24" t="s">
-        <v>494</v>
       </c>
       <c r="M3" s="24">
         <v>4</v>
       </c>
       <c r="N3" s="24" t="s">
+        <v>494</v>
+      </c>
+      <c r="O3" s="24" t="s">
         <v>495</v>
-      </c>
-      <c r="O3" s="24" t="s">
-        <v>496</v>
       </c>
       <c r="P3" s="24">
         <v>1</v>
       </c>
       <c r="Q3" s="24" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="R3" s="24" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -4829,16 +4829,16 @@
         <v>467</v>
       </c>
       <c r="B4" s="24" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="C4" s="38" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="D4" s="24">
         <v>2</v>
       </c>
       <c r="E4" s="38" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="F4" s="25">
         <v>2</v>
@@ -4847,16 +4847,16 @@
         <v>3</v>
       </c>
       <c r="H4" s="24" t="s">
+        <v>489</v>
+      </c>
+      <c r="I4" s="24" t="s">
         <v>490</v>
       </c>
-      <c r="I4" s="24" t="s">
+      <c r="J4" s="24" t="s">
         <v>491</v>
       </c>
-      <c r="J4" s="24" t="s">
-        <v>492</v>
-      </c>
       <c r="K4" s="24" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="L4" s="24"/>
       <c r="M4" s="24"/>
@@ -4892,7 +4892,7 @@
     </row>
     <row r="13" spans="1:18">
       <c r="D13" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="E13" s="51"/>
     </row>
@@ -7681,7 +7681,7 @@
   <sheetData>
     <row r="1" spans="1:30" s="1" customFormat="1" ht="93" customHeight="1">
       <c r="A1" s="59" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="B1" s="60"/>
       <c r="C1" s="60"/>
@@ -7718,67 +7718,67 @@
         <v>0</v>
       </c>
       <c r="B2" s="47" t="s">
+        <v>473</v>
+      </c>
+      <c r="C2" s="48" t="s">
         <v>474</v>
       </c>
-      <c r="C2" s="48" t="s">
-        <v>475</v>
-      </c>
       <c r="D2" s="48" t="s">
+        <v>500</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>529</v>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>530</v>
+      </c>
+      <c r="G2" s="47" t="s">
         <v>501</v>
       </c>
-      <c r="E2" s="7" t="s">
-        <v>530</v>
-      </c>
-      <c r="F2" s="7" t="s">
-        <v>531</v>
-      </c>
-      <c r="G2" s="47" t="s">
+      <c r="H2" s="47" t="s">
         <v>502</v>
-      </c>
-      <c r="H2" s="47" t="s">
-        <v>503</v>
       </c>
       <c r="I2" s="48" t="s">
         <v>179</v>
       </c>
       <c r="J2" s="47" t="s">
+        <v>503</v>
+      </c>
+      <c r="K2" s="47" t="s">
         <v>504</v>
       </c>
-      <c r="K2" s="47" t="s">
+      <c r="L2" s="47" t="s">
         <v>505</v>
       </c>
-      <c r="L2" s="47" t="s">
+      <c r="M2" s="47" t="s">
         <v>506</v>
       </c>
-      <c r="M2" s="47" t="s">
+      <c r="N2" s="47" t="s">
         <v>507</v>
       </c>
-      <c r="N2" s="47" t="s">
+      <c r="O2" s="47" t="s">
+        <v>521</v>
+      </c>
+      <c r="P2" s="47" t="s">
+        <v>522</v>
+      </c>
+      <c r="Q2" s="47" t="s">
+        <v>525</v>
+      </c>
+      <c r="R2" s="47" t="s">
+        <v>515</v>
+      </c>
+      <c r="S2" s="47" t="s">
+        <v>516</v>
+      </c>
+      <c r="T2" s="47" t="s">
         <v>508</v>
       </c>
-      <c r="O2" s="47" t="s">
-        <v>522</v>
-      </c>
-      <c r="P2" s="47" t="s">
-        <v>523</v>
-      </c>
-      <c r="Q2" s="47" t="s">
-        <v>526</v>
-      </c>
-      <c r="R2" s="47" t="s">
-        <v>516</v>
-      </c>
-      <c r="S2" s="47" t="s">
+      <c r="U2" s="47" t="s">
+        <v>509</v>
+      </c>
+      <c r="V2" s="47" t="s">
         <v>517</v>
-      </c>
-      <c r="T2" s="47" t="s">
-        <v>509</v>
-      </c>
-      <c r="U2" s="47" t="s">
-        <v>510</v>
-      </c>
-      <c r="V2" s="47" t="s">
-        <v>518</v>
       </c>
       <c r="W2" s="53" t="s">
         <v>461</v>
@@ -7796,22 +7796,22 @@
         <v>467</v>
       </c>
       <c r="B3" s="24" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="C3" s="38" t="s">
+        <v>510</v>
+      </c>
+      <c r="D3" s="24" t="s">
         <v>511</v>
       </c>
-      <c r="D3" s="24" t="s">
+      <c r="E3" s="25" t="s">
+        <v>535</v>
+      </c>
+      <c r="F3" s="25" t="s">
+        <v>533</v>
+      </c>
+      <c r="G3" s="25" t="s">
         <v>512</v>
-      </c>
-      <c r="E3" s="25" t="s">
-        <v>536</v>
-      </c>
-      <c r="F3" s="25" t="s">
-        <v>534</v>
-      </c>
-      <c r="G3" s="25" t="s">
-        <v>513</v>
       </c>
       <c r="H3" s="24">
         <v>4</v>
@@ -7820,10 +7820,10 @@
         <v>225</v>
       </c>
       <c r="J3" s="38" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="K3" s="38" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="L3" s="38">
         <v>914</v>
@@ -7835,10 +7835,10 @@
         <v>96</v>
       </c>
       <c r="O3" s="38" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="P3" s="56" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="Q3" s="56"/>
       <c r="R3" s="38" t="b">
@@ -7848,16 +7848,16 @@
         <v>0</v>
       </c>
       <c r="T3" s="38" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="U3" s="55" t="s">
+        <v>513</v>
+      </c>
+      <c r="V3" s="55" t="s">
+        <v>518</v>
+      </c>
+      <c r="W3" s="25" t="s">
         <v>514</v>
-      </c>
-      <c r="V3" s="55" t="s">
-        <v>519</v>
-      </c>
-      <c r="W3" s="25" t="s">
-        <v>515</v>
       </c>
     </row>
     <row r="4" spans="1:30" ht="48">
@@ -7865,22 +7865,22 @@
         <v>467</v>
       </c>
       <c r="B4" s="24" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="C4" s="38" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="D4" s="24" t="s">
+        <v>536</v>
+      </c>
+      <c r="E4" s="25" t="s">
         <v>537</v>
       </c>
-      <c r="E4" s="25" t="s">
+      <c r="F4" s="25" t="s">
         <v>538</v>
       </c>
-      <c r="F4" s="25" t="s">
-        <v>539</v>
-      </c>
       <c r="G4" s="25" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="H4" s="24">
         <v>4</v>
@@ -7889,10 +7889,10 @@
         <v>225</v>
       </c>
       <c r="J4" s="38" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="K4" s="38" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="L4" s="38">
         <v>914</v>
@@ -7904,10 +7904,10 @@
         <v>96</v>
       </c>
       <c r="O4" s="38" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="P4" s="56" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="Q4" s="56"/>
       <c r="R4" s="38" t="b">
@@ -7917,16 +7917,16 @@
         <v>0</v>
       </c>
       <c r="T4" s="38" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="U4" s="55" t="s">
+        <v>513</v>
+      </c>
+      <c r="V4" s="55" t="s">
+        <v>518</v>
+      </c>
+      <c r="W4" s="25" t="s">
         <v>514</v>
-      </c>
-      <c r="V4" s="55" t="s">
-        <v>519</v>
-      </c>
-      <c r="W4" s="25" t="s">
-        <v>515</v>
       </c>
     </row>
     <row r="5" spans="1:30">

</xml_diff>